<commit_message>
feat: implement client-side app logic, payroll handling, and date utilities
</commit_message>
<xml_diff>
--- a/payroll/APADAMI -SALARY SHEET -SEP 2026.xlsx
+++ b/payroll/APADAMI -SALARY SHEET -SEP 2026.xlsx
@@ -207,7 +207,7 @@
     <ns0:t>17 D</ns0:t>
   </ns0:si>
   <ns0:si>
-    <ns0:t>SALARY SHEET  (IN GBP ) -SEPTEMBER 2026 </ns0:t>
+    <ns0:t>SALARY SHEET (IN GBP) - SEPTEMBER 2026</ns0:t>
   </ns0:si>
   <ns0:si>
     <ns0:t>908114167V</ns0:t>
@@ -216,7 +216,7 @@
     <ns0:t>703-020085698 (HNB)</ns0:t>
   </ns0:si>
   <ns0:si>
-    <ns0:t>SALARY SHEET  (IN GBP ) -SEPTEMBER2026. @440</ns0:t>
+    <ns0:t>SALARY SHEET (IN LKR) - SEPTEMBER 2026 @ 440</ns0:t>
   </ns0:si>
   <ns0:si>
     <ns0:t>15.04.2026</ns0:t>

</xml_diff>